<commit_message>
Update results and upload presentation file
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws\git-workspaces\github-com\build-stuff-jmeter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F7B1AEA-759A-4F6D-A4AF-3E5A88917B57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36C8EF2-79F2-4C78-925A-4F29C3F95CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2190" yWindow="2220" windowWidth="21600" windowHeight="12645" xr2:uid="{7E9936F2-0EA3-480D-A3CE-C60916FDE704}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7E9936F2-0EA3-480D-A3CE-C60916FDE704}"/>
   </bookViews>
   <sheets>
     <sheet name="Demo app" sheetId="1" r:id="rId1"/>
@@ -732,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F6C6E9-C61A-46FB-862D-AB8C861E3A0B}">
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -908,7 +908,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="13" t="b">
-        <f t="shared" ref="B5:B11" si="0">OR(C5&lt;C$2,D5&lt;D$2,E5&lt;E$2,D5&lt;D$2,F5&lt;F$2,G5&lt;G$2,H5&lt;H$2,I5&lt;I$2,J5&lt;J$2,K5&lt;K$2,L5&lt;L$2,M5&lt;M$2,N5&lt;N$2,O5&lt;O$2)</f>
+        <f t="shared" ref="B5:B12" si="0">OR(C5&lt;C$2,D5&lt;D$2,E5&lt;E$2,D5&lt;D$2,F5&lt;F$2,G5&lt;G$2,H5&lt;H$2,I5&lt;I$2,J5&lt;J$2,K5&lt;K$2,L5&lt;L$2,M5&lt;M$2,N5&lt;N$2,O5&lt;O$2)</f>
         <v>1</v>
       </c>
       <c r="C5" s="1">
@@ -1196,7 +1196,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="13" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B11" si="1">OR(C11&lt;C$2,D11&lt;D$2,E11&lt;E$2,D11&lt;D$2,F11&lt;F$2,G11&lt;G$2,H11&lt;H$2,I11&lt;I$2,J11&lt;J$2,K11&lt;K$2,L11&lt;L$2,M11&lt;M$2,N11&lt;N$2,O11&lt;O$2)</f>
         <v>1</v>
       </c>
       <c r="C11" s="1">
@@ -1240,124 +1240,172 @@
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="6"/>
-      <c r="B12" s="13"/>
-      <c r="J12" s="6"/>
-      <c r="O12" s="6"/>
+      <c r="A12" s="6">
+        <v>7</v>
+      </c>
+      <c r="B12" s="13" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>478</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2.82</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.84</v>
+      </c>
+      <c r="F12" s="1">
+        <v>537</v>
+      </c>
+      <c r="G12" s="1">
+        <v>535</v>
+      </c>
+      <c r="H12" s="1">
+        <v>166</v>
+      </c>
+      <c r="I12" s="1">
+        <v>1.71</v>
+      </c>
+      <c r="J12" s="6">
+        <v>522</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="L12" s="1">
+        <v>1.74</v>
+      </c>
+      <c r="M12" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.72</v>
+      </c>
+      <c r="O12" s="6">
+        <v>1.53</v>
+      </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="B13" s="18"/>
-      <c r="C13" s="11">
-        <f>AVERAGE(C5:C12)</f>
-        <v>419.57142857142856</v>
-      </c>
-      <c r="D13" s="11">
-        <f t="shared" ref="D13:O13" si="1">AVERAGE(D5:D12)</f>
-        <v>2.3971428571428572</v>
-      </c>
-      <c r="E13" s="11">
-        <f t="shared" si="1"/>
-        <v>0.85857142857142854</v>
-      </c>
-      <c r="F13" s="11">
-        <f t="shared" si="1"/>
-        <v>522.57142857142856</v>
-      </c>
-      <c r="G13" s="11">
-        <f t="shared" si="1"/>
-        <v>527.57142857142856</v>
-      </c>
-      <c r="H13" s="11">
-        <f t="shared" si="1"/>
-        <v>165.71428571428572</v>
-      </c>
-      <c r="I13" s="11">
-        <f t="shared" si="1"/>
-        <v>1.6800000000000002</v>
-      </c>
-      <c r="J13" s="11">
-        <f t="shared" si="1"/>
-        <v>515.57142857142856</v>
-      </c>
-      <c r="K13" s="11">
-        <f t="shared" si="1"/>
-        <v>1.8385714285714285</v>
-      </c>
-      <c r="L13" s="11">
-        <f t="shared" si="1"/>
-        <v>1.8314285714285714</v>
-      </c>
-      <c r="M13" s="11">
-        <f t="shared" si="1"/>
-        <v>1.7614285714285713</v>
-      </c>
-      <c r="N13" s="11">
-        <f t="shared" si="1"/>
-        <v>1.6814285714285713</v>
-      </c>
-      <c r="O13" s="12">
-        <f t="shared" si="1"/>
-        <v>1.4857142857142858</v>
-      </c>
+      <c r="A13" s="6"/>
+      <c r="B13" s="13"/>
+      <c r="J13" s="6"/>
+      <c r="O13" s="6"/>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B14" s="20"/>
+      <c r="A14" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="18"/>
       <c r="C14" s="11">
-        <f>MIN(C5:C12)</f>
-        <v>347</v>
+        <f>AVERAGE(C5:C13)</f>
+        <v>426.875</v>
       </c>
       <c r="D14" s="11">
-        <f t="shared" ref="D14:O14" si="2">MIN(D5:D12)</f>
-        <v>1.5</v>
+        <f t="shared" ref="D14:O14" si="2">AVERAGE(D5:D13)</f>
+        <v>2.4500000000000002</v>
       </c>
       <c r="E14" s="11">
         <f t="shared" si="2"/>
-        <v>0.8</v>
+        <v>0.85624999999999996</v>
       </c>
       <c r="F14" s="11">
         <f t="shared" si="2"/>
-        <v>454</v>
+        <v>524.375</v>
       </c>
       <c r="G14" s="11">
         <f t="shared" si="2"/>
-        <v>443</v>
+        <v>528.5</v>
       </c>
       <c r="H14" s="11">
         <f t="shared" si="2"/>
-        <v>165</v>
+        <v>165.75</v>
       </c>
       <c r="I14" s="11">
         <f t="shared" si="2"/>
-        <v>1.5</v>
+        <v>1.6837500000000003</v>
       </c>
       <c r="J14" s="11">
         <f t="shared" si="2"/>
-        <v>436</v>
+        <v>516.375</v>
       </c>
       <c r="K14" s="11">
         <f t="shared" si="2"/>
-        <v>1.72</v>
+        <v>1.8274999999999999</v>
       </c>
       <c r="L14" s="11">
         <f t="shared" si="2"/>
-        <v>1.7</v>
+        <v>1.82</v>
       </c>
       <c r="M14" s="11">
         <f t="shared" si="2"/>
-        <v>1.68</v>
+        <v>1.7662500000000001</v>
       </c>
       <c r="N14" s="11">
         <f t="shared" si="2"/>
-        <v>1.65</v>
+        <v>1.68625</v>
       </c>
       <c r="O14" s="12">
         <f t="shared" si="2"/>
+        <v>1.49125</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" s="20"/>
+      <c r="C15" s="11">
+        <f>MIN(C5:C13)</f>
+        <v>347</v>
+      </c>
+      <c r="D15" s="11">
+        <f t="shared" ref="D15:O15" si="3">MIN(D5:D13)</f>
+        <v>1.5</v>
+      </c>
+      <c r="E15" s="11">
+        <f t="shared" si="3"/>
+        <v>0.8</v>
+      </c>
+      <c r="F15" s="11">
+        <f t="shared" si="3"/>
+        <v>454</v>
+      </c>
+      <c r="G15" s="11">
+        <f t="shared" si="3"/>
+        <v>443</v>
+      </c>
+      <c r="H15" s="11">
+        <f t="shared" si="3"/>
+        <v>165</v>
+      </c>
+      <c r="I15" s="11">
+        <f t="shared" si="3"/>
+        <v>1.5</v>
+      </c>
+      <c r="J15" s="11">
+        <f t="shared" si="3"/>
+        <v>436</v>
+      </c>
+      <c r="K15" s="11">
+        <f t="shared" si="3"/>
+        <v>1.72</v>
+      </c>
+      <c r="L15" s="11">
+        <f t="shared" si="3"/>
+        <v>1.7</v>
+      </c>
+      <c r="M15" s="11">
+        <f t="shared" si="3"/>
+        <v>1.68</v>
+      </c>
+      <c r="N15" s="11">
+        <f t="shared" si="3"/>
+        <v>1.65</v>
+      </c>
+      <c r="O15" s="12">
+        <f t="shared" si="3"/>
         <v>1.42</v>
       </c>
     </row>
@@ -1365,13 +1413,13 @@
   <mergeCells count="7">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="K1:O1"/>
-    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C3:J3"/>
     <mergeCell ref="K3:O3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B11">
+  <conditionalFormatting sqref="B5:B12">
     <cfRule type="cellIs" dxfId="3" priority="14" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
@@ -1379,7 +1427,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:O11">
+  <conditionalFormatting sqref="C5:O12">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>C$2</formula>
     </cfRule>

</xml_diff>

<commit_message>
Disable push trigger, update results
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws\git-workspaces\github-com\build-stuff-jmeter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B36C8EF2-79F2-4C78-925A-4F29C3F95CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0534B20A-B35A-4544-9C49-AEADC933E070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7E9936F2-0EA3-480D-A3CE-C60916FDE704}"/>
+    <workbookView xWindow="3855" yWindow="3855" windowWidth="28800" windowHeight="15345" xr2:uid="{7E9936F2-0EA3-480D-A3CE-C60916FDE704}"/>
   </bookViews>
   <sheets>
     <sheet name="Demo app" sheetId="1" r:id="rId1"/>
@@ -732,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F6C6E9-C61A-46FB-862D-AB8C861E3A0B}">
-  <dimension ref="A1:O15"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -908,7 +908,7 @@
         <v>1</v>
       </c>
       <c r="B5" s="13" t="b">
-        <f t="shared" ref="B5:B12" si="0">OR(C5&lt;C$2,D5&lt;D$2,E5&lt;E$2,D5&lt;D$2,F5&lt;F$2,G5&lt;G$2,H5&lt;H$2,I5&lt;I$2,J5&lt;J$2,K5&lt;K$2,L5&lt;L$2,M5&lt;M$2,N5&lt;N$2,O5&lt;O$2)</f>
+        <f t="shared" ref="B5:B13" si="0">OR(C5&lt;C$2,D5&lt;D$2,E5&lt;E$2,D5&lt;D$2,F5&lt;F$2,G5&lt;G$2,H5&lt;H$2,I5&lt;I$2,J5&lt;J$2,K5&lt;K$2,L5&lt;L$2,M5&lt;M$2,N5&lt;N$2,O5&lt;O$2)</f>
         <v>1</v>
       </c>
       <c r="C5" s="1">
@@ -1196,7 +1196,7 @@
         <v>6</v>
       </c>
       <c r="B11" s="13" t="b">
-        <f t="shared" ref="B11" si="1">OR(C11&lt;C$2,D11&lt;D$2,E11&lt;E$2,D11&lt;D$2,F11&lt;F$2,G11&lt;G$2,H11&lt;H$2,I11&lt;I$2,J11&lt;J$2,K11&lt;K$2,L11&lt;L$2,M11&lt;M$2,N11&lt;N$2,O11&lt;O$2)</f>
+        <f t="shared" ref="B11:B12" si="1">OR(C11&lt;C$2,D11&lt;D$2,E11&lt;E$2,D11&lt;D$2,F11&lt;F$2,G11&lt;G$2,H11&lt;H$2,I11&lt;I$2,J11&lt;J$2,K11&lt;K$2,L11&lt;L$2,M11&lt;M$2,N11&lt;N$2,O11&lt;O$2)</f>
         <v>1</v>
       </c>
       <c r="C11" s="1">
@@ -1244,167 +1244,215 @@
         <v>7</v>
       </c>
       <c r="B12" s="13" t="b">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C12" s="1">
+        <v>478</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2.82</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.84</v>
+      </c>
+      <c r="F12" s="1">
+        <v>537</v>
+      </c>
+      <c r="G12" s="1">
+        <v>535</v>
+      </c>
+      <c r="H12" s="1">
+        <v>166</v>
+      </c>
+      <c r="I12" s="1">
+        <v>1.71</v>
+      </c>
+      <c r="J12" s="6">
+        <v>522</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="L12" s="1">
+        <v>1.74</v>
+      </c>
+      <c r="M12" s="1">
+        <v>1.8</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.72</v>
+      </c>
+      <c r="O12" s="6">
+        <v>1.53</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" s="6">
+        <v>8</v>
+      </c>
+      <c r="B13" s="13" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="C12" s="1">
-        <v>478</v>
-      </c>
-      <c r="D12" s="1">
-        <v>2.82</v>
-      </c>
-      <c r="E12" s="1">
-        <v>0.84</v>
-      </c>
-      <c r="F12" s="1">
-        <v>537</v>
-      </c>
-      <c r="G12" s="1">
-        <v>535</v>
-      </c>
-      <c r="H12" s="1">
+      <c r="C13" s="1">
+        <v>540</v>
+      </c>
+      <c r="D13" s="1">
+        <v>2.86</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0.89</v>
+      </c>
+      <c r="F13" s="1">
+        <v>595</v>
+      </c>
+      <c r="G13" s="1">
+        <v>602</v>
+      </c>
+      <c r="H13" s="1">
         <v>166</v>
       </c>
-      <c r="I12" s="1">
+      <c r="I13" s="1">
         <v>1.71</v>
       </c>
-      <c r="J12" s="6">
-        <v>522</v>
-      </c>
-      <c r="K12" s="1">
-        <v>1.75</v>
-      </c>
-      <c r="L12" s="1">
+      <c r="J13" s="6">
+        <v>596</v>
+      </c>
+      <c r="K13" s="1">
         <v>1.74</v>
       </c>
-      <c r="M12" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="N12" s="1">
-        <v>1.72</v>
-      </c>
-      <c r="O12" s="6">
-        <v>1.53</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="6"/>
-      <c r="B13" s="13"/>
-      <c r="J13" s="6"/>
-      <c r="O13" s="6"/>
+      <c r="L13" s="1">
+        <v>1.73</v>
+      </c>
+      <c r="M13" s="1">
+        <v>1.73</v>
+      </c>
+      <c r="N13" s="1">
+        <v>1.63</v>
+      </c>
+      <c r="O13" s="6">
+        <v>1.44</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="6"/>
+      <c r="B14" s="13"/>
+      <c r="J14" s="6"/>
+      <c r="O14" s="6"/>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="18"/>
-      <c r="C14" s="11">
-        <f>AVERAGE(C5:C13)</f>
-        <v>426.875</v>
-      </c>
-      <c r="D14" s="11">
-        <f t="shared" ref="D14:O14" si="2">AVERAGE(D5:D13)</f>
-        <v>2.4500000000000002</v>
-      </c>
-      <c r="E14" s="11">
+      <c r="B15" s="18"/>
+      <c r="C15" s="11">
+        <f>AVERAGE(C5:C14)</f>
+        <v>439.44444444444446</v>
+      </c>
+      <c r="D15" s="11">
+        <f>AVERAGE(D5:D14)</f>
+        <v>2.4955555555555557</v>
+      </c>
+      <c r="E15" s="11">
+        <f t="shared" ref="D15:O15" si="2">AVERAGE(E5:E14)</f>
+        <v>0.85999999999999988</v>
+      </c>
+      <c r="F15" s="11">
         <f t="shared" si="2"/>
-        <v>0.85624999999999996</v>
-      </c>
-      <c r="F14" s="11">
+        <v>532.22222222222217</v>
+      </c>
+      <c r="G15" s="11">
         <f t="shared" si="2"/>
-        <v>524.375</v>
-      </c>
-      <c r="G14" s="11">
+        <v>536.66666666666663</v>
+      </c>
+      <c r="H15" s="11">
         <f t="shared" si="2"/>
-        <v>528.5</v>
-      </c>
-      <c r="H14" s="11">
+        <v>165.77777777777777</v>
+      </c>
+      <c r="I15" s="11">
         <f t="shared" si="2"/>
-        <v>165.75</v>
-      </c>
-      <c r="I14" s="11">
+        <v>1.686666666666667</v>
+      </c>
+      <c r="J15" s="11">
         <f t="shared" si="2"/>
-        <v>1.6837500000000003</v>
-      </c>
-      <c r="J14" s="11">
+        <v>525.22222222222217</v>
+      </c>
+      <c r="K15" s="11">
         <f t="shared" si="2"/>
-        <v>516.375</v>
-      </c>
-      <c r="K14" s="11">
+        <v>1.8177777777777777</v>
+      </c>
+      <c r="L15" s="11">
         <f t="shared" si="2"/>
-        <v>1.8274999999999999</v>
-      </c>
-      <c r="L14" s="11">
+        <v>1.8099999999999998</v>
+      </c>
+      <c r="M15" s="11">
         <f t="shared" si="2"/>
-        <v>1.82</v>
-      </c>
-      <c r="M14" s="11">
+        <v>1.7622222222222224</v>
+      </c>
+      <c r="N15" s="11">
         <f t="shared" si="2"/>
-        <v>1.7662500000000001</v>
-      </c>
-      <c r="N14" s="11">
+        <v>1.6800000000000002</v>
+      </c>
+      <c r="O15" s="12">
         <f t="shared" si="2"/>
-        <v>1.68625</v>
-      </c>
-      <c r="O14" s="12">
-        <f t="shared" si="2"/>
-        <v>1.49125</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="19" t="s">
+        <v>1.4855555555555555</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="20"/>
-      <c r="C15" s="11">
-        <f>MIN(C5:C13)</f>
+      <c r="B16" s="20"/>
+      <c r="C16" s="11">
+        <f>MIN(C5:C14)</f>
         <v>347</v>
       </c>
-      <c r="D15" s="11">
-        <f t="shared" ref="D15:O15" si="3">MIN(D5:D13)</f>
+      <c r="D16" s="11">
+        <f t="shared" ref="D16:O16" si="3">MIN(D5:D14)</f>
         <v>1.5</v>
       </c>
-      <c r="E15" s="11">
+      <c r="E16" s="11">
         <f t="shared" si="3"/>
         <v>0.8</v>
       </c>
-      <c r="F15" s="11">
+      <c r="F16" s="11">
         <f t="shared" si="3"/>
         <v>454</v>
       </c>
-      <c r="G15" s="11">
+      <c r="G16" s="11">
         <f t="shared" si="3"/>
         <v>443</v>
       </c>
-      <c r="H15" s="11">
+      <c r="H16" s="11">
         <f t="shared" si="3"/>
         <v>165</v>
       </c>
-      <c r="I15" s="11">
+      <c r="I16" s="11">
         <f t="shared" si="3"/>
         <v>1.5</v>
       </c>
-      <c r="J15" s="11">
+      <c r="J16" s="11">
         <f t="shared" si="3"/>
         <v>436</v>
       </c>
-      <c r="K15" s="11">
+      <c r="K16" s="11">
         <f t="shared" si="3"/>
         <v>1.72</v>
       </c>
-      <c r="L15" s="11">
+      <c r="L16" s="11">
         <f t="shared" si="3"/>
         <v>1.7</v>
       </c>
-      <c r="M15" s="11">
+      <c r="M16" s="11">
         <f t="shared" si="3"/>
         <v>1.68</v>
       </c>
-      <c r="N15" s="11">
+      <c r="N16" s="11">
         <f t="shared" si="3"/>
-        <v>1.65</v>
-      </c>
-      <c r="O15" s="12">
+        <v>1.63</v>
+      </c>
+      <c r="O16" s="12">
         <f t="shared" si="3"/>
         <v>1.42</v>
       </c>
@@ -1413,13 +1461,13 @@
   <mergeCells count="7">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="K1:O1"/>
-    <mergeCell ref="A14:B14"/>
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A16:B16"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C3:J3"/>
     <mergeCell ref="K3:O3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B12">
+  <conditionalFormatting sqref="B5:B13">
     <cfRule type="cellIs" dxfId="3" priority="14" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
@@ -1427,7 +1475,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:O12">
+  <conditionalFormatting sqref="C5:O13">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>C$2</formula>
     </cfRule>

</xml_diff>

<commit_message>
Update ppt and results excel
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws\git-workspaces\github-com\build-stuff-jmeter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0534B20A-B35A-4544-9C49-AEADC933E070}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D11568F-F2CA-404C-AA70-4885224F341C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3855" yWindow="3855" windowWidth="28800" windowHeight="15345" xr2:uid="{7E9936F2-0EA3-480D-A3CE-C60916FDE704}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7E9936F2-0EA3-480D-A3CE-C60916FDE704}"/>
   </bookViews>
   <sheets>
     <sheet name="Demo app" sheetId="1" r:id="rId1"/>
@@ -732,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F6C6E9-C61A-46FB-862D-AB8C861E3A0B}">
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -759,31 +759,31 @@
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="2">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="D1" s="2">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="E1" s="2">
+        <v>40</v>
+      </c>
+      <c r="F1" s="2">
         <v>45</v>
       </c>
-      <c r="F1" s="2">
-        <v>60</v>
-      </c>
       <c r="G1" s="2">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="H1" s="2">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="I1" s="2">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="J1" s="8">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="K1" s="15">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="L1" s="14"/>
       <c r="M1" s="14"/>
@@ -796,7 +796,7 @@
       </c>
       <c r="B2" s="14"/>
       <c r="C2" s="2">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="D2" s="2">
         <v>2</v>
@@ -805,10 +805,10 @@
         <v>0.8</v>
       </c>
       <c r="F2" s="2">
-        <v>510</v>
+        <v>300</v>
       </c>
       <c r="G2" s="2">
-        <v>520</v>
+        <v>320</v>
       </c>
       <c r="H2" s="2">
         <v>150</v>
@@ -817,7 +817,7 @@
         <v>1.5</v>
       </c>
       <c r="J2" s="8">
-        <v>510</v>
+        <v>330</v>
       </c>
       <c r="K2" s="2">
         <v>1.6</v>
@@ -908,44 +908,44 @@
         <v>1</v>
       </c>
       <c r="B5" s="13" t="b">
-        <f t="shared" ref="B5:B13" si="0">OR(C5&lt;C$2,D5&lt;D$2,E5&lt;E$2,D5&lt;D$2,F5&lt;F$2,G5&lt;G$2,H5&lt;H$2,I5&lt;I$2,J5&lt;J$2,K5&lt;K$2,L5&lt;L$2,M5&lt;M$2,N5&lt;N$2,O5&lt;O$2)</f>
-        <v>1</v>
+        <f t="shared" ref="B5:B6" si="0">OR(C5&lt;C$2,D5&lt;D$2,E5&lt;E$2,D5&lt;D$2,F5&lt;F$2,G5&lt;G$2,H5&lt;H$2,I5&lt;I$2,J5&lt;J$2,K5&lt;K$2,L5&lt;L$2,M5&lt;M$2,N5&lt;N$2,O5&lt;O$2)</f>
+        <v>0</v>
       </c>
       <c r="C5" s="1">
-        <v>347</v>
+        <v>340</v>
       </c>
       <c r="D5" s="1">
-        <v>2.1800000000000002</v>
+        <v>2.5</v>
       </c>
       <c r="E5" s="1">
-        <v>0.87</v>
+        <v>0.8</v>
       </c>
       <c r="F5" s="1">
-        <v>603</v>
+        <v>301</v>
       </c>
       <c r="G5" s="1">
-        <v>607</v>
+        <v>325</v>
       </c>
       <c r="H5" s="1">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="I5" s="1">
-        <v>1.69</v>
+        <v>1.55</v>
       </c>
       <c r="J5" s="6">
-        <v>594</v>
+        <v>335</v>
       </c>
       <c r="K5" s="1">
-        <v>2.17</v>
+        <v>1.6</v>
       </c>
       <c r="L5" s="1">
-        <v>1.9</v>
+        <v>1.62</v>
       </c>
       <c r="M5" s="1">
-        <v>1.68</v>
+        <v>1.63</v>
       </c>
       <c r="N5" s="1">
-        <v>1.66</v>
+        <v>1.6</v>
       </c>
       <c r="O5" s="6">
         <v>1.42</v>
@@ -957,46 +957,46 @@
       </c>
       <c r="B6" s="13" t="b">
         <f t="shared" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6" s="1">
-        <v>386</v>
+        <v>345</v>
       </c>
       <c r="D6" s="1">
-        <v>1.5</v>
+        <v>3.04</v>
       </c>
       <c r="E6" s="1">
         <v>0.87</v>
       </c>
       <c r="F6" s="1">
-        <v>602</v>
+        <v>344</v>
       </c>
       <c r="G6" s="1">
-        <v>602</v>
+        <v>334</v>
       </c>
       <c r="H6" s="1">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="I6" s="1">
+        <v>1.69</v>
+      </c>
+      <c r="J6" s="6">
+        <v>340</v>
+      </c>
+      <c r="K6" s="1">
         <v>1.75</v>
       </c>
-      <c r="J6" s="6">
-        <v>590</v>
-      </c>
-      <c r="K6" s="1">
-        <v>1.87</v>
-      </c>
       <c r="L6" s="1">
-        <v>1.92</v>
+        <v>1.77</v>
       </c>
       <c r="M6" s="1">
-        <v>1.85</v>
+        <v>1.72</v>
       </c>
       <c r="N6" s="1">
         <v>1.69</v>
       </c>
       <c r="O6" s="6">
-        <v>1.53</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
@@ -1004,143 +1004,143 @@
         <v>3</v>
       </c>
       <c r="B7" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>0</v>
+        <f t="shared" ref="B7" si="1">OR(C7&lt;C$2,D7&lt;D$2,E7&lt;E$2,D7&lt;D$2,F7&lt;F$2,G7&lt;G$2,H7&lt;H$2,I7&lt;I$2,J7&lt;J$2,K7&lt;K$2,L7&lt;L$2,M7&lt;M$2,N7&lt;N$2,O7&lt;O$2)</f>
+        <v>1</v>
       </c>
       <c r="C7" s="1">
-        <v>488</v>
+        <v>291</v>
       </c>
       <c r="D7" s="1">
-        <v>2.84</v>
+        <v>3.02</v>
       </c>
       <c r="E7" s="1">
-        <v>0.88</v>
+        <v>0.84</v>
       </c>
       <c r="F7" s="1">
-        <v>536</v>
+        <v>288</v>
       </c>
       <c r="G7" s="1">
-        <v>582</v>
+        <v>269</v>
       </c>
       <c r="H7" s="1">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="I7" s="1">
-        <v>1.74</v>
+        <v>1.73</v>
       </c>
       <c r="J7" s="6">
-        <v>530</v>
+        <v>288</v>
       </c>
       <c r="K7" s="1">
-        <v>1.72</v>
+        <v>1.78</v>
       </c>
       <c r="L7" s="1">
-        <v>1.7</v>
+        <v>1.75</v>
       </c>
       <c r="M7" s="1">
-        <v>1.69</v>
+        <v>1.75</v>
       </c>
       <c r="N7" s="1">
         <v>1.67</v>
       </c>
       <c r="O7" s="6">
-        <v>1.44</v>
+        <v>1.57</v>
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B8" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" ref="B8:B10" si="2">OR(C8&lt;C$2,D8&lt;D$2,E8&lt;E$2,D8&lt;D$2,F8&lt;F$2,G8&lt;G$2,H8&lt;H$2,I8&lt;I$2,J8&lt;J$2,K8&lt;K$2,L8&lt;L$2,M8&lt;M$2,N8&lt;N$2,O8&lt;O$2)</f>
+        <v>0</v>
       </c>
       <c r="C8" s="1">
-        <v>424</v>
+        <v>354</v>
       </c>
       <c r="D8" s="1">
-        <v>2.89</v>
+        <v>3.13</v>
       </c>
       <c r="E8" s="1">
-        <v>0.8</v>
+        <v>0.85</v>
       </c>
       <c r="F8" s="1">
-        <v>476</v>
+        <v>343</v>
       </c>
       <c r="G8" s="1">
-        <v>462</v>
+        <v>330</v>
       </c>
       <c r="H8" s="1">
         <v>166</v>
       </c>
       <c r="I8" s="1">
-        <v>1.71</v>
+        <v>1.69</v>
       </c>
       <c r="J8" s="6">
-        <v>466</v>
+        <v>340</v>
       </c>
       <c r="K8" s="1">
+        <v>1.78</v>
+      </c>
+      <c r="L8" s="1">
+        <v>1.73</v>
+      </c>
+      <c r="M8" s="1">
         <v>1.77</v>
       </c>
-      <c r="L8" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="M8" s="1">
-        <v>1.76</v>
-      </c>
       <c r="N8" s="1">
-        <v>1.65</v>
+        <v>1.68</v>
       </c>
       <c r="O8" s="6">
-        <v>1.48</v>
+        <v>1.58</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B9" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
+        <f t="shared" ref="B9" si="3">OR(C9&lt;C$2,D9&lt;D$2,E9&lt;E$2,D9&lt;D$2,F9&lt;F$2,G9&lt;G$2,H9&lt;H$2,I9&lt;I$2,J9&lt;J$2,K9&lt;K$2,L9&lt;L$2,M9&lt;M$2,N9&lt;N$2,O9&lt;O$2)</f>
+        <v>0</v>
       </c>
       <c r="C9" s="1">
-        <v>422</v>
+        <v>427</v>
       </c>
       <c r="D9" s="1">
-        <v>1.75</v>
+        <v>3.1</v>
       </c>
       <c r="E9" s="1">
         <v>0.88</v>
       </c>
       <c r="F9" s="1">
-        <v>474</v>
+        <v>421</v>
       </c>
       <c r="G9" s="1">
-        <v>468</v>
+        <v>412</v>
       </c>
       <c r="H9" s="1">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I9" s="1">
-        <v>1.5</v>
+        <v>1.69</v>
       </c>
       <c r="J9" s="6">
-        <v>467</v>
+        <v>419</v>
       </c>
       <c r="K9" s="1">
-        <v>1.81</v>
+        <v>1.77</v>
       </c>
       <c r="L9" s="1">
-        <v>1.8</v>
+        <v>1.75</v>
       </c>
       <c r="M9" s="1">
-        <v>1.84</v>
+        <v>1.73</v>
       </c>
       <c r="N9" s="1">
-        <v>1.68</v>
+        <v>1.69</v>
       </c>
       <c r="O9" s="6">
-        <v>1.51</v>
+        <v>1.63</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
@@ -1148,312 +1148,168 @@
         <v>5</v>
       </c>
       <c r="B10" s="13" t="b">
-        <f t="shared" si="0"/>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="C10" s="1">
-        <v>474</v>
+        <v>469</v>
       </c>
       <c r="D10" s="1">
-        <v>2.86</v>
+        <v>3.11</v>
       </c>
       <c r="E10" s="1">
         <v>0.87</v>
       </c>
       <c r="F10" s="1">
-        <v>513</v>
+        <v>481</v>
       </c>
       <c r="G10" s="1">
-        <v>529</v>
+        <v>474</v>
       </c>
       <c r="H10" s="1">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I10" s="1">
-        <v>1.66</v>
+        <v>1.68</v>
       </c>
       <c r="J10" s="6">
-        <v>526</v>
+        <v>481</v>
       </c>
       <c r="K10" s="1">
         <v>1.76</v>
       </c>
       <c r="L10" s="1">
-        <v>1.91</v>
+        <v>1.83</v>
       </c>
       <c r="M10" s="1">
-        <v>1.77</v>
+        <v>1.73</v>
       </c>
       <c r="N10" s="1">
         <v>1.72</v>
       </c>
       <c r="O10" s="6">
-        <v>1.52</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="6">
-        <v>6</v>
-      </c>
-      <c r="B11" s="13" t="b">
-        <f t="shared" ref="B11:B12" si="1">OR(C11&lt;C$2,D11&lt;D$2,E11&lt;E$2,D11&lt;D$2,F11&lt;F$2,G11&lt;G$2,H11&lt;H$2,I11&lt;I$2,J11&lt;J$2,K11&lt;K$2,L11&lt;L$2,M11&lt;M$2,N11&lt;N$2,O11&lt;O$2)</f>
-        <v>1</v>
-      </c>
-      <c r="C11" s="1">
-        <v>396</v>
-      </c>
-      <c r="D11" s="1">
-        <v>2.76</v>
-      </c>
-      <c r="E11" s="1">
-        <v>0.84</v>
-      </c>
-      <c r="F11" s="1">
-        <v>454</v>
-      </c>
-      <c r="G11" s="1">
-        <v>443</v>
-      </c>
-      <c r="H11" s="1">
-        <v>166</v>
-      </c>
-      <c r="I11" s="1">
-        <v>1.71</v>
-      </c>
-      <c r="J11" s="6">
-        <v>436</v>
-      </c>
-      <c r="K11" s="1">
-        <v>1.77</v>
-      </c>
-      <c r="L11" s="1">
-        <v>1.82</v>
-      </c>
-      <c r="M11" s="1">
-        <v>1.74</v>
-      </c>
-      <c r="N11" s="1">
-        <v>1.7</v>
-      </c>
-      <c r="O11" s="6">
-        <v>1.5</v>
-      </c>
+      <c r="A11" s="6"/>
+      <c r="B11" s="13"/>
+      <c r="J11" s="6"/>
+      <c r="O11" s="6"/>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="6">
-        <v>7</v>
-      </c>
-      <c r="B12" s="13" t="b">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="C12" s="1">
-        <v>478</v>
-      </c>
-      <c r="D12" s="1">
-        <v>2.82</v>
-      </c>
-      <c r="E12" s="1">
-        <v>0.84</v>
-      </c>
-      <c r="F12" s="1">
-        <v>537</v>
-      </c>
-      <c r="G12" s="1">
-        <v>535</v>
-      </c>
-      <c r="H12" s="1">
-        <v>166</v>
-      </c>
-      <c r="I12" s="1">
-        <v>1.71</v>
-      </c>
-      <c r="J12" s="6">
-        <v>522</v>
-      </c>
-      <c r="K12" s="1">
-        <v>1.75</v>
-      </c>
-      <c r="L12" s="1">
+      <c r="A12" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" s="18"/>
+      <c r="C12" s="11">
+        <f>AVERAGE(C5:C11)</f>
+        <v>371</v>
+      </c>
+      <c r="D12" s="11">
+        <f>AVERAGE(D5:D11)</f>
+        <v>2.9833333333333338</v>
+      </c>
+      <c r="E12" s="11">
+        <f>AVERAGE(E5:E11)</f>
+        <v>0.85166666666666668</v>
+      </c>
+      <c r="F12" s="11">
+        <f>AVERAGE(F5:F11)</f>
+        <v>363</v>
+      </c>
+      <c r="G12" s="11">
+        <f>AVERAGE(G5:G11)</f>
+        <v>357.33333333333331</v>
+      </c>
+      <c r="H12" s="11">
+        <f>AVERAGE(H5:H11)</f>
+        <v>164</v>
+      </c>
+      <c r="I12" s="11">
+        <f>AVERAGE(I5:I11)</f>
+        <v>1.6716666666666666</v>
+      </c>
+      <c r="J12" s="11">
+        <f>AVERAGE(J5:J11)</f>
+        <v>367.16666666666669</v>
+      </c>
+      <c r="K12" s="11">
+        <f>AVERAGE(K5:K11)</f>
         <v>1.74</v>
       </c>
-      <c r="M12" s="1">
-        <v>1.8</v>
-      </c>
-      <c r="N12" s="1">
-        <v>1.72</v>
-      </c>
-      <c r="O12" s="6">
-        <v>1.53</v>
+      <c r="L12" s="11">
+        <f>AVERAGE(L5:L11)</f>
+        <v>1.7416666666666669</v>
+      </c>
+      <c r="M12" s="11">
+        <f>AVERAGE(M5:M11)</f>
+        <v>1.7216666666666667</v>
+      </c>
+      <c r="N12" s="11">
+        <f>AVERAGE(N5:N11)</f>
+        <v>1.675</v>
+      </c>
+      <c r="O12" s="12">
+        <f>AVERAGE(O5:O11)</f>
+        <v>1.5633333333333335</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="6">
-        <v>8</v>
-      </c>
-      <c r="B13" s="13" t="b">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C13" s="1">
-        <v>540</v>
-      </c>
-      <c r="D13" s="1">
-        <v>2.86</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0.89</v>
-      </c>
-      <c r="F13" s="1">
-        <v>595</v>
-      </c>
-      <c r="G13" s="1">
-        <v>602</v>
-      </c>
-      <c r="H13" s="1">
-        <v>166</v>
-      </c>
-      <c r="I13" s="1">
-        <v>1.71</v>
-      </c>
-      <c r="J13" s="6">
-        <v>596</v>
-      </c>
-      <c r="K13" s="1">
-        <v>1.74</v>
-      </c>
-      <c r="L13" s="1">
-        <v>1.73</v>
-      </c>
-      <c r="M13" s="1">
-        <v>1.73</v>
-      </c>
-      <c r="N13" s="1">
+      <c r="A13" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="B13" s="20"/>
+      <c r="C13" s="11">
+        <f>MIN(C5:C11)</f>
+        <v>291</v>
+      </c>
+      <c r="D13" s="11">
+        <f>MIN(D5:D11)</f>
+        <v>2.5</v>
+      </c>
+      <c r="E13" s="11">
+        <f>MIN(E5:E11)</f>
+        <v>0.8</v>
+      </c>
+      <c r="F13" s="11">
+        <f>MIN(F5:F11)</f>
+        <v>288</v>
+      </c>
+      <c r="G13" s="11">
+        <f>MIN(G5:G11)</f>
+        <v>269</v>
+      </c>
+      <c r="H13" s="11">
+        <f>MIN(H5:H11)</f>
+        <v>158</v>
+      </c>
+      <c r="I13" s="11">
+        <f>MIN(I5:I11)</f>
+        <v>1.55</v>
+      </c>
+      <c r="J13" s="11">
+        <f>MIN(J5:J11)</f>
+        <v>288</v>
+      </c>
+      <c r="K13" s="11">
+        <f>MIN(K5:K11)</f>
+        <v>1.6</v>
+      </c>
+      <c r="L13" s="11">
+        <f>MIN(L5:L11)</f>
+        <v>1.62</v>
+      </c>
+      <c r="M13" s="11">
+        <f>MIN(M5:M11)</f>
         <v>1.63</v>
       </c>
-      <c r="O13" s="6">
-        <v>1.44</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A14" s="6"/>
-      <c r="B14" s="13"/>
-      <c r="J14" s="6"/>
-      <c r="O14" s="6"/>
-    </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A15" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="B15" s="18"/>
-      <c r="C15" s="11">
-        <f>AVERAGE(C5:C14)</f>
-        <v>439.44444444444446</v>
-      </c>
-      <c r="D15" s="11">
-        <f>AVERAGE(D5:D14)</f>
-        <v>2.4955555555555557</v>
-      </c>
-      <c r="E15" s="11">
-        <f t="shared" ref="D15:O15" si="2">AVERAGE(E5:E14)</f>
-        <v>0.85999999999999988</v>
-      </c>
-      <c r="F15" s="11">
-        <f t="shared" si="2"/>
-        <v>532.22222222222217</v>
-      </c>
-      <c r="G15" s="11">
-        <f t="shared" si="2"/>
-        <v>536.66666666666663</v>
-      </c>
-      <c r="H15" s="11">
-        <f t="shared" si="2"/>
-        <v>165.77777777777777</v>
-      </c>
-      <c r="I15" s="11">
-        <f t="shared" si="2"/>
-        <v>1.686666666666667</v>
-      </c>
-      <c r="J15" s="11">
-        <f t="shared" si="2"/>
-        <v>525.22222222222217</v>
-      </c>
-      <c r="K15" s="11">
-        <f t="shared" si="2"/>
-        <v>1.8177777777777777</v>
-      </c>
-      <c r="L15" s="11">
-        <f t="shared" si="2"/>
-        <v>1.8099999999999998</v>
-      </c>
-      <c r="M15" s="11">
-        <f t="shared" si="2"/>
-        <v>1.7622222222222224</v>
-      </c>
-      <c r="N15" s="11">
-        <f t="shared" si="2"/>
-        <v>1.6800000000000002</v>
-      </c>
-      <c r="O15" s="12">
-        <f t="shared" si="2"/>
-        <v>1.4855555555555555</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A16" s="19" t="s">
-        <v>14</v>
-      </c>
-      <c r="B16" s="20"/>
-      <c r="C16" s="11">
-        <f>MIN(C5:C14)</f>
-        <v>347</v>
-      </c>
-      <c r="D16" s="11">
-        <f t="shared" ref="D16:O16" si="3">MIN(D5:D14)</f>
-        <v>1.5</v>
-      </c>
-      <c r="E16" s="11">
-        <f t="shared" si="3"/>
-        <v>0.8</v>
-      </c>
-      <c r="F16" s="11">
-        <f t="shared" si="3"/>
-        <v>454</v>
-      </c>
-      <c r="G16" s="11">
-        <f t="shared" si="3"/>
-        <v>443</v>
-      </c>
-      <c r="H16" s="11">
-        <f t="shared" si="3"/>
-        <v>165</v>
-      </c>
-      <c r="I16" s="11">
-        <f t="shared" si="3"/>
-        <v>1.5</v>
-      </c>
-      <c r="J16" s="11">
-        <f t="shared" si="3"/>
-        <v>436</v>
-      </c>
-      <c r="K16" s="11">
-        <f t="shared" si="3"/>
-        <v>1.72</v>
-      </c>
-      <c r="L16" s="11">
-        <f t="shared" si="3"/>
-        <v>1.7</v>
-      </c>
-      <c r="M16" s="11">
-        <f t="shared" si="3"/>
-        <v>1.68</v>
-      </c>
-      <c r="N16" s="11">
-        <f t="shared" si="3"/>
-        <v>1.63</v>
-      </c>
-      <c r="O16" s="12">
-        <f t="shared" si="3"/>
+      <c r="N13" s="11">
+        <f>MIN(N5:N11)</f>
+        <v>1.6</v>
+      </c>
+      <c r="O13" s="12">
+        <f>MIN(O5:O11)</f>
         <v>1.42</v>
       </c>
     </row>
@@ -1461,13 +1317,13 @@
   <mergeCells count="7">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="K1:O1"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:B16"/>
+    <mergeCell ref="A12:B12"/>
+    <mergeCell ref="A13:B13"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C3:J3"/>
     <mergeCell ref="K3:O3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B13">
+  <conditionalFormatting sqref="B5:B10">
     <cfRule type="cellIs" dxfId="3" priority="14" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
@@ -1475,7 +1331,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:O13">
+  <conditionalFormatting sqref="C5:O10">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>C$2</formula>
     </cfRule>

</xml_diff>

<commit_message>
Update tests and results and latest ppt
</commit_message>
<xml_diff>
--- a/results.xlsx
+++ b/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ws\git-workspaces\github-com\build-stuff-jmeter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D11568F-F2CA-404C-AA70-4885224F341C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443CA620-4CAB-48EF-8C44-6889ACEA4291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{7E9936F2-0EA3-480D-A3CE-C60916FDE704}"/>
   </bookViews>
@@ -732,7 +732,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39F6C6E9-C61A-46FB-862D-AB8C861E3A0B}">
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:O15"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.85546875" style="1" bestFit="1" customWidth="1"/>
@@ -759,31 +759,31 @@
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="2">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="D1" s="2">
-        <v>140</v>
+        <v>120</v>
       </c>
       <c r="E1" s="2">
         <v>40</v>
       </c>
       <c r="F1" s="2">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G1" s="2">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="H1" s="2">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="I1" s="2">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="J1" s="8">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="K1" s="15">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="L1" s="14"/>
       <c r="M1" s="14"/>
@@ -1052,7 +1052,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="13" t="b">
-        <f t="shared" ref="B8:B10" si="2">OR(C8&lt;C$2,D8&lt;D$2,E8&lt;E$2,D8&lt;D$2,F8&lt;F$2,G8&lt;G$2,H8&lt;H$2,I8&lt;I$2,J8&lt;J$2,K8&lt;K$2,L8&lt;L$2,M8&lt;M$2,N8&lt;N$2,O8&lt;O$2)</f>
+        <f t="shared" ref="B8:B12" si="2">OR(C8&lt;C$2,D8&lt;D$2,E8&lt;E$2,D8&lt;D$2,F8&lt;F$2,G8&lt;G$2,H8&lt;H$2,I8&lt;I$2,J8&lt;J$2,K8&lt;K$2,L8&lt;L$2,M8&lt;M$2,N8&lt;N$2,O8&lt;O$2)</f>
         <v>0</v>
       </c>
       <c r="C8" s="1">
@@ -1100,7 +1100,7 @@
         <v>5</v>
       </c>
       <c r="B9" s="13" t="b">
-        <f t="shared" ref="B9" si="3">OR(C9&lt;C$2,D9&lt;D$2,E9&lt;E$2,D9&lt;D$2,F9&lt;F$2,G9&lt;G$2,H9&lt;H$2,I9&lt;I$2,J9&lt;J$2,K9&lt;K$2,L9&lt;L$2,M9&lt;M$2,N9&lt;N$2,O9&lt;O$2)</f>
+        <f t="shared" ref="B9:B11" si="3">OR(C9&lt;C$2,D9&lt;D$2,E9&lt;E$2,D9&lt;D$2,F9&lt;F$2,G9&lt;G$2,H9&lt;H$2,I9&lt;I$2,J9&lt;J$2,K9&lt;K$2,L9&lt;L$2,M9&lt;M$2,N9&lt;N$2,O9&lt;O$2)</f>
         <v>0</v>
       </c>
       <c r="C9" s="1">
@@ -1145,171 +1145,267 @@
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" s="6">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B10" s="13" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="C10" s="1">
+        <v>469</v>
+      </c>
+      <c r="D10" s="1">
+        <v>3.11</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0.87</v>
+      </c>
+      <c r="F10" s="1">
+        <v>481</v>
+      </c>
+      <c r="G10" s="1">
+        <v>474</v>
+      </c>
+      <c r="H10" s="1">
+        <v>167</v>
+      </c>
+      <c r="I10" s="1">
+        <v>1.68</v>
+      </c>
+      <c r="J10" s="6">
+        <v>481</v>
+      </c>
+      <c r="K10" s="1">
+        <v>1.76</v>
+      </c>
+      <c r="L10" s="1">
+        <v>1.83</v>
+      </c>
+      <c r="M10" s="1">
+        <v>1.73</v>
+      </c>
+      <c r="N10" s="1">
+        <v>1.72</v>
+      </c>
+      <c r="O10" s="6">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" s="6">
+        <v>7</v>
+      </c>
+      <c r="B11" s="13" t="b">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="C11" s="1">
+        <v>415</v>
+      </c>
+      <c r="D11" s="1">
+        <v>3.01</v>
+      </c>
+      <c r="E11" s="1">
+        <v>0.87</v>
+      </c>
+      <c r="F11" s="1">
+        <v>432</v>
+      </c>
+      <c r="G11" s="1">
+        <v>425</v>
+      </c>
+      <c r="H11" s="1">
+        <v>167</v>
+      </c>
+      <c r="I11" s="1">
+        <v>1.7</v>
+      </c>
+      <c r="J11" s="6">
+        <v>431</v>
+      </c>
+      <c r="K11" s="1">
+        <v>1.79</v>
+      </c>
+      <c r="L11" s="1">
+        <v>1.78</v>
+      </c>
+      <c r="M11" s="1">
+        <v>1.75</v>
+      </c>
+      <c r="N11" s="1">
+        <v>1.68</v>
+      </c>
+      <c r="O11" s="6">
+        <v>1.52</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" s="6">
+        <v>8</v>
+      </c>
+      <c r="B12" s="13" t="b">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="C10" s="1">
-        <v>469</v>
-      </c>
-      <c r="D10" s="1">
-        <v>3.11</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0.87</v>
-      </c>
-      <c r="F10" s="1">
-        <v>481</v>
-      </c>
-      <c r="G10" s="1">
-        <v>474</v>
-      </c>
-      <c r="H10" s="1">
+      <c r="C12" s="1">
+        <v>362</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2.96</v>
+      </c>
+      <c r="E12" s="1">
+        <v>0.86</v>
+      </c>
+      <c r="F12" s="1">
+        <v>377</v>
+      </c>
+      <c r="G12" s="1">
+        <v>371</v>
+      </c>
+      <c r="H12" s="1">
         <v>167</v>
       </c>
-      <c r="I10" s="1">
-        <v>1.68</v>
-      </c>
-      <c r="J10" s="6">
-        <v>481</v>
-      </c>
-      <c r="K10" s="1">
-        <v>1.76</v>
-      </c>
-      <c r="L10" s="1">
+      <c r="I12" s="1">
+        <v>1.71</v>
+      </c>
+      <c r="J12" s="6">
+        <v>378</v>
+      </c>
+      <c r="K12" s="1">
+        <v>1.94</v>
+      </c>
+      <c r="L12" s="1">
         <v>1.83</v>
       </c>
-      <c r="M10" s="1">
-        <v>1.73</v>
-      </c>
-      <c r="N10" s="1">
-        <v>1.72</v>
-      </c>
-      <c r="O10" s="6">
-        <v>1.6</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A11" s="6"/>
-      <c r="B11" s="13"/>
-      <c r="J11" s="6"/>
-      <c r="O11" s="6"/>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A12" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="11">
-        <f>AVERAGE(C5:C11)</f>
-        <v>371</v>
-      </c>
-      <c r="D12" s="11">
-        <f>AVERAGE(D5:D11)</f>
-        <v>2.9833333333333338</v>
-      </c>
-      <c r="E12" s="11">
-        <f>AVERAGE(E5:E11)</f>
-        <v>0.85166666666666668</v>
-      </c>
-      <c r="F12" s="11">
-        <f>AVERAGE(F5:F11)</f>
-        <v>363</v>
-      </c>
-      <c r="G12" s="11">
-        <f>AVERAGE(G5:G11)</f>
-        <v>357.33333333333331</v>
-      </c>
-      <c r="H12" s="11">
-        <f>AVERAGE(H5:H11)</f>
-        <v>164</v>
-      </c>
-      <c r="I12" s="11">
-        <f>AVERAGE(I5:I11)</f>
-        <v>1.6716666666666666</v>
-      </c>
-      <c r="J12" s="11">
-        <f>AVERAGE(J5:J11)</f>
-        <v>367.16666666666669</v>
-      </c>
-      <c r="K12" s="11">
-        <f>AVERAGE(K5:K11)</f>
-        <v>1.74</v>
-      </c>
-      <c r="L12" s="11">
-        <f>AVERAGE(L5:L11)</f>
-        <v>1.7416666666666669</v>
-      </c>
-      <c r="M12" s="11">
-        <f>AVERAGE(M5:M11)</f>
-        <v>1.7216666666666667</v>
-      </c>
-      <c r="N12" s="11">
-        <f>AVERAGE(N5:N11)</f>
-        <v>1.675</v>
-      </c>
-      <c r="O12" s="12">
-        <f>AVERAGE(O5:O11)</f>
-        <v>1.5633333333333335</v>
+      <c r="M12" s="1">
+        <v>1.79</v>
+      </c>
+      <c r="N12" s="1">
+        <v>1.69</v>
+      </c>
+      <c r="O12" s="6">
+        <v>1.59</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A13" s="19" t="s">
+      <c r="A13" s="6"/>
+      <c r="B13" s="13"/>
+      <c r="J13" s="6"/>
+      <c r="O13" s="6"/>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" s="18"/>
+      <c r="C14" s="11">
+        <f t="shared" ref="C14:O14" si="4">AVERAGE(C5:C13)</f>
+        <v>375.375</v>
+      </c>
+      <c r="D14" s="11">
+        <f t="shared" si="4"/>
+        <v>2.9837500000000006</v>
+      </c>
+      <c r="E14" s="11">
+        <f t="shared" si="4"/>
+        <v>0.85500000000000009</v>
+      </c>
+      <c r="F14" s="11">
+        <f t="shared" si="4"/>
+        <v>373.375</v>
+      </c>
+      <c r="G14" s="11">
+        <f t="shared" si="4"/>
+        <v>367.5</v>
+      </c>
+      <c r="H14" s="11">
+        <f t="shared" si="4"/>
+        <v>164.75</v>
+      </c>
+      <c r="I14" s="11">
+        <f t="shared" si="4"/>
+        <v>1.6799999999999997</v>
+      </c>
+      <c r="J14" s="11">
+        <f t="shared" si="4"/>
+        <v>376.5</v>
+      </c>
+      <c r="K14" s="11">
+        <f t="shared" si="4"/>
+        <v>1.77125</v>
+      </c>
+      <c r="L14" s="11">
+        <f t="shared" si="4"/>
+        <v>1.7575000000000001</v>
+      </c>
+      <c r="M14" s="11">
+        <f t="shared" si="4"/>
+        <v>1.7337500000000001</v>
+      </c>
+      <c r="N14" s="11">
+        <f t="shared" si="4"/>
+        <v>1.6775</v>
+      </c>
+      <c r="O14" s="12">
+        <f t="shared" si="4"/>
+        <v>1.56125</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="B13" s="20"/>
-      <c r="C13" s="11">
-        <f>MIN(C5:C11)</f>
+      <c r="B15" s="20"/>
+      <c r="C15" s="11">
+        <f t="shared" ref="C15:O15" si="5">MIN(C5:C13)</f>
         <v>291</v>
       </c>
-      <c r="D13" s="11">
-        <f>MIN(D5:D11)</f>
+      <c r="D15" s="11">
+        <f t="shared" si="5"/>
         <v>2.5</v>
       </c>
-      <c r="E13" s="11">
-        <f>MIN(E5:E11)</f>
+      <c r="E15" s="11">
+        <f t="shared" si="5"/>
         <v>0.8</v>
       </c>
-      <c r="F13" s="11">
-        <f>MIN(F5:F11)</f>
+      <c r="F15" s="11">
+        <f t="shared" si="5"/>
         <v>288</v>
       </c>
-      <c r="G13" s="11">
-        <f>MIN(G5:G11)</f>
+      <c r="G15" s="11">
+        <f t="shared" si="5"/>
         <v>269</v>
       </c>
-      <c r="H13" s="11">
-        <f>MIN(H5:H11)</f>
+      <c r="H15" s="11">
+        <f t="shared" si="5"/>
         <v>158</v>
       </c>
-      <c r="I13" s="11">
-        <f>MIN(I5:I11)</f>
+      <c r="I15" s="11">
+        <f t="shared" si="5"/>
         <v>1.55</v>
       </c>
-      <c r="J13" s="11">
-        <f>MIN(J5:J11)</f>
+      <c r="J15" s="11">
+        <f t="shared" si="5"/>
         <v>288</v>
       </c>
-      <c r="K13" s="11">
-        <f>MIN(K5:K11)</f>
+      <c r="K15" s="11">
+        <f t="shared" si="5"/>
         <v>1.6</v>
       </c>
-      <c r="L13" s="11">
-        <f>MIN(L5:L11)</f>
+      <c r="L15" s="11">
+        <f t="shared" si="5"/>
         <v>1.62</v>
       </c>
-      <c r="M13" s="11">
-        <f>MIN(M5:M11)</f>
+      <c r="M15" s="11">
+        <f t="shared" si="5"/>
         <v>1.63</v>
       </c>
-      <c r="N13" s="11">
-        <f>MIN(N5:N11)</f>
+      <c r="N15" s="11">
+        <f t="shared" si="5"/>
         <v>1.6</v>
       </c>
-      <c r="O13" s="12">
-        <f>MIN(O5:O11)</f>
+      <c r="O15" s="12">
+        <f t="shared" si="5"/>
         <v>1.42</v>
       </c>
     </row>
@@ -1317,13 +1413,13 @@
   <mergeCells count="7">
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="K1:O1"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:B13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="A15:B15"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="C3:J3"/>
     <mergeCell ref="K3:O3"/>
   </mergeCells>
-  <conditionalFormatting sqref="B5:B10">
+  <conditionalFormatting sqref="B5:B12">
     <cfRule type="cellIs" dxfId="3" priority="14" operator="equal">
       <formula>FALSE</formula>
     </cfRule>
@@ -1331,7 +1427,7 @@
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C5:O10">
+  <conditionalFormatting sqref="C5:O12">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>C$2</formula>
     </cfRule>

</xml_diff>